<commit_message>
update 25_12 short reading
</commit_message>
<xml_diff>
--- a/READING/8_25_12.xlsx
+++ b/READING/8_25_12.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\N2_2025_12\READING\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52DB9837-33F2-45A5-A28D-B6E6FA96BDBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C924E71C-8CAD-454A-B1AD-913C266FC3F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10710" yWindow="630" windowWidth="20880" windowHeight="19995" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19800" yWindow="1440" windowWidth="20880" windowHeight="19995" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="92">
   <si>
     <t>Fre</t>
   </si>
@@ -37,13 +37,433 @@
   </si>
   <si>
     <t>备注</t>
+  </si>
+  <si>
+    <t>いいます</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>「言う」的ます</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>こちら</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>我们；本公司;这里；这位</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>なければ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>如果不...的话</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>口にする</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>说出</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ふうに</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>样子，方式</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>まま</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>状态持续</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>では</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>假设</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>よう</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>意志，提议</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>てもらえる</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>もらう可能态</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>自分へ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>对自己</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>問いかけ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>询问</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>よりよい</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>更好的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>なっておりま</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>す</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>(1)正在变得…(2)正处于…状态</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>原型「なっている」，</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>「おる」是「いる」</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>的自谦</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>これらの</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>这些</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>市</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>市政府，市区</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>目印</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>标记；标志；记号</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>为了…；对于…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>には</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>対応できません</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>无法处理</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>つくり手</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>生产者</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>つくる制作</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>売り買い</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>买卖、交易</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>何よりも</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>最重要地…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>～のである</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>是…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>出来</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>做好;完成</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>振り返る</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>回顾、反思</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>～のか</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>是否</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>といった</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>…之类的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>それぞれ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>每个;各自</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>やり取り</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>交换；交流；对话</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>やる</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>-&gt;做</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>届く</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>收到；到达；</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ていただく</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>「てもらう」</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>敬语</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>見積もり書</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>报价单</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>見積</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>估计，估算</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>代金</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>货款</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>とは別に</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>除此之外还有</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>設置</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>安装;设立</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>～のうえ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>动作先后</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ふつう</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>通常、一般</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>どういうときに</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>在什么时候？</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>はずだ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>应该；理应；预期</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>したがって</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>从而、因此</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>あるとかないとか</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>有啊、没有啊之类的</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>決して～ない</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>无论如何也不…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -52,17 +472,48 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <sz val="9"/>
       <name val="宋体"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Yu Gothic"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="128"/>
     </font>
   </fonts>
   <fills count="2">
@@ -100,10 +551,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -407,14 +867,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="9" customWidth="1"/>
-    <col min="2" max="2" width="17.875" customWidth="1"/>
-    <col min="3" max="3" width="23.75" customWidth="1"/>
-    <col min="4" max="4" width="10.375" customWidth="1"/>
-    <col min="5" max="5" width="9" customWidth="1"/>
+    <col min="1" max="1" width="9" style="2" customWidth="1"/>
+    <col min="2" max="2" width="17.875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="23.75" style="2" customWidth="1"/>
+    <col min="4" max="4" width="10.375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="12.625" style="2" customWidth="1"/>
+    <col min="6" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.15">
@@ -434,8 +895,479 @@
         <v>4</v>
       </c>
     </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A2" s="2">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A3" s="2">
+        <v>0</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A4" s="2">
+        <v>0</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A5" s="2">
+        <v>0</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A6" s="2">
+        <v>0</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A7" s="2">
+        <v>0</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A8" s="2">
+        <v>0</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A9" s="2">
+        <v>0</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A10" s="2">
+        <v>0</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A11" s="2">
+        <v>0</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A12" s="2">
+        <v>0</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A13" s="2">
+        <v>0</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A14" s="2">
+        <v>0</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A15" s="2">
+        <v>0</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A16" s="2">
+        <v>0</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A17" s="2">
+        <v>0</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A18" s="2">
+        <v>0</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A19" s="2">
+        <v>0</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A20" s="2">
+        <v>0</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A21" s="2">
+        <v>0</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A22" s="2">
+        <v>0</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A23" s="2">
+        <v>0</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A24" s="2">
+        <v>0</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A25" s="2">
+        <v>0</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A26" s="2">
+        <v>0</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A27" s="2">
+        <v>0</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A28" s="2">
+        <v>0</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A29" s="2">
+        <v>0</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A30" s="2">
+        <v>0</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A31" s="2">
+        <v>0</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A32" s="2">
+        <v>0</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A33" s="2">
+        <v>0</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A34" s="2">
+        <v>0</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A35" s="2">
+        <v>0</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A36" s="2">
+        <v>0</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A37" s="2">
+        <v>0</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A38" s="2">
+        <v>0</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A39" s="2">
+        <v>0</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A40" s="2">
+        <v>0</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A41" s="2">
+        <v>0</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A42" s="2">
+        <v>0</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A43" s="2">
+        <v>0</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -446,7 +1378,7 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <sheetData/>
-  <phoneticPr fontId="2" type="noConversion"/>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -456,7 +1388,7 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <sheetData/>
-  <phoneticPr fontId="2" type="noConversion"/>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>